<commit_message>
[refactor] UIBase 재설계 / 로직 분리
[추가]
- 수학 계산 관련 로직을 (MathUtility)정적 클래스로 옮김
- Planet의 스폰 위치를 결정하는 계산기 클래스 추가, Spawn은 이제 스폰 시점, 스폰 목록 등만 관리
[수정]
- OnEnable/OnDisable 직접 구독 → RegisterEvents/UnregisterEvents 오버라이드 방식으로 통일
- 데이터 주입 메서드를 Setup(object data)로 일원화
- Open/Close 생명주기를 UIBase에서 관리, OnBeforeClose로 정리 시점 제어
- StationUpgrade.Open(zoneType, station) → Setup(StationUpgradeData)로 통일
- UIManager OpenUI/CloseUI → UIBase.Open/Close 경유하도록 변경
</commit_message>
<xml_diff>
--- a/JsonConverter/ExcelFiles/Planet.xlsx
+++ b/JsonConverter/ExcelFiles/Planet.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11520" windowHeight="9000"/>
+    <workbookView windowWidth="13272" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -87,7 +87,7 @@
     <t>BaseOre</t>
   </si>
   <si>
-    <t>Property</t>
+    <t>Properity</t>
   </si>
   <si>
     <t>Grade</t>
@@ -1632,7 +1632,7 @@
         <v>18000</v>
       </c>
       <c r="E5">
-        <f t="shared" ref="E5:E25" si="0">ROUND(D5/1000,0)*2</f>
+        <f t="shared" ref="E5:E27" si="0">ROUND(D5/1000,0)*2</f>
         <v>36</v>
       </c>
       <c r="F5">
@@ -2262,7 +2262,7 @@
         <v>530000</v>
       </c>
       <c r="E26">
-        <f>ROUND(D26/1000,0)*2</f>
+        <f t="shared" si="0"/>
         <v>1060</v>
       </c>
       <c r="F26">
@@ -2292,7 +2292,7 @@
         <v>565000</v>
       </c>
       <c r="E27">
-        <f>ROUND(D27/1000,0)*2</f>
+        <f t="shared" si="0"/>
         <v>1130</v>
       </c>
       <c r="F27">

</xml_diff>